<commit_message>
feat: add PLC command acknowledgement and heartbeat
</commit_message>
<xml_diff>
--- a/outputs/2026-08-23-tia-v18-point-list-v1/PLC-POINT-LIST-V1.xlsx
+++ b/outputs/2026-08-23-tia-v18-point-list-v1/PLC-POINT-LIST-V1.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="点表V1" sheetId="1" r:id="R636f1b6c7b6f46ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" r:id="Rc5fba8c5966441d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="点表V1" sheetId="1" r:id="Rdd838d857df441bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" r:id="R3838813369e642d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -444,14 +444,14 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="3">
+  <x:dxfs count="4">
     <x:dxf>
       <x:font>
         <x:b/>
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -461,7 +461,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -471,8 +471,19 @@
         <x:color rgb="FF595959"/>
       </x:font>
       <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE7E6E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1F4E78"/>
+      </x:font>
+      <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE7E6E6"/>
+          <x:bgColor rgb="FFDDEBF7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -1116,10 +1127,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I13" s="29" t="str">
-        <x:v>命令流水号；后续用于请求/应答去重</x:v>
+        <x:v>命令流水号；用于请求/应答去重</x:v>
       </x:c>
       <x:c r="J13" s="28" t="str">
-        <x:v>已预留</x:v>
+        <x:v>条件启用</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
@@ -1151,7 +1162,7 @@
         <x:v>上位机心跳递增计数</x:v>
       </x:c>
       <x:c r="J14" s="28" t="str">
-        <x:v>已预留</x:v>
+        <x:v>条件启用</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
@@ -1183,7 +1194,7 @@
         <x:v>通信协议主版本号，V1 固定为 1</x:v>
       </x:c>
       <x:c r="J15" s="28" t="str">
-        <x:v>已预留</x:v>
+        <x:v>已使用</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
@@ -1215,7 +1226,7 @@
         <x:v>上位机已连接且业务服务就绪</x:v>
       </x:c>
       <x:c r="J16" s="28" t="str">
-        <x:v>已预留</x:v>
+        <x:v>已使用</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
@@ -1631,7 +1642,7 @@
         <x:v>PLC 已处理的命令流水号</x:v>
       </x:c>
       <x:c r="J29" s="28" t="str">
-        <x:v>已预留</x:v>
+        <x:v>条件启用</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
@@ -1727,7 +1738,7 @@
         <x:v>PLC 心跳递增计数</x:v>
       </x:c>
       <x:c r="J32" s="28" t="str">
-        <x:v>已预留</x:v>
+        <x:v>条件启用</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
@@ -1759,7 +1770,7 @@
         <x:v>PLC 实现的通信协议主版本号</x:v>
       </x:c>
       <x:c r="J33" s="28" t="str">
-        <x:v>已预留</x:v>
+        <x:v>已使用</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="24" customHeight="1">
@@ -1791,7 +1802,7 @@
         <x:v>PLC 正在处理上位机命令</x:v>
       </x:c>
       <x:c r="J34" s="28" t="str">
-        <x:v>已预留</x:v>
+        <x:v>条件启用</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="24" customHeight="1">
@@ -1823,7 +1834,7 @@
         <x:v>最近一次上位机命令处理失败</x:v>
       </x:c>
       <x:c r="J35" s="28" t="str">
-        <x:v>已预留</x:v>
+        <x:v>条件启用</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="24" customHeight="1">
@@ -2079,7 +2090,7 @@
         <x:v>最近一次命令结果；0成功，非0错误码</x:v>
       </x:c>
       <x:c r="J43" s="30" t="str">
-        <x:v>已预留</x:v>
+        <x:v>条件启用</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2087,10 +2098,11 @@
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="已使用"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="已预留"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="未使用"/>
+    <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="条件启用"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6937f75df67647a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re40ea8f44803401d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2174,7 +2186,7 @@
         <x:v>当前限制</x:v>
       </x:c>
       <x:c r="B10" s="71" t="str">
-        <x:v>命令序号、应答与心跳已预留，但完整握手逻辑尚未启用</x:v>
+        <x:v>C# 已实现可配置应答与心跳；PLC 处理逻辑和 TIA 编译尚未完成</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>